<commit_message>
commit changes for 2024 rookies
</commit_message>
<xml_diff>
--- a/2020 Rookies/2020_Rookie_Profiles.xlsx
+++ b/2020 Rookies/2020_Rookie_Profiles.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bborh\OneDrive - The Ohio State University\Fantasy Football\Rookie Ranking\2020 Rookies\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bborh\Documents\Fantasy Football\Rookie Ranking\2020 Rookies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B9A7A2F-3521-4CF6-9080-E7DB7F52D380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B11249A0-DE46-419A-AA99-3FDF3ABA60A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10148" yWindow="-98" windowWidth="19395" windowHeight="11596" activeTab="2" xr2:uid="{039B20E9-F581-4683-903F-646ADA475269}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{039B20E9-F581-4683-903F-646ADA475269}"/>
   </bookViews>
   <sheets>
     <sheet name="Quarterbacks" sheetId="1" r:id="rId1"/>
@@ -507,7 +507,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -522,7 +522,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -530,7 +529,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -895,7 +893,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{19196FA0-4F4A-48D1-9010-8C077D45CF45}" name="Table3" displayName="Table3" ref="A1:AB21" totalsRowShown="0" headerRowDxfId="19">
   <autoFilter ref="A1:AB21" xr:uid="{19196FA0-4F4A-48D1-9010-8C077D45CF45}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AB21">
-    <sortCondition ref="D2:D21"/>
+    <sortCondition ref="C1:C21"/>
   </sortState>
   <tableColumns count="28">
     <tableColumn id="1" xr3:uid="{D2DD26F2-3A1D-4E48-8E9B-7588005BC91E}" name="Player" dataDxfId="18"/>
@@ -1242,82 +1240,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="13" t="s">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="K1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="L1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="M1" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="N1" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="O1" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="P1" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="Q1" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="R1" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="S1" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="T1" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="U1" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="V1" s="13" t="s">
+      <c r="V1" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="W1" s="13" t="s">
+      <c r="W1" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="X1" s="13" t="s">
+      <c r="X1" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="Y1" s="13" t="s">
+      <c r="Y1" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="Z1" s="13" t="s">
+      <c r="Z1" s="11" t="s">
         <v>126</v>
       </c>
     </row>
@@ -1379,19 +1377,19 @@
       </c>
       <c r="S2" s="4">
         <f ca="1">(TODAY()-R2)/365-1</f>
-        <v>24.358904109589041</v>
-      </c>
-      <c r="T2" s="11">
+        <v>26.402739726027399</v>
+      </c>
+      <c r="T2" s="10">
         <f>6*12+4</f>
         <v>76</v>
       </c>
-      <c r="U2" s="11">
+      <c r="U2" s="10">
         <v>221</v>
       </c>
-      <c r="V2" s="11">
+      <c r="V2" s="10">
         <v>10</v>
       </c>
-      <c r="W2" s="11">
+      <c r="W2" s="10">
         <v>709</v>
       </c>
       <c r="X2" s="4">
@@ -1401,7 +1399,7 @@
         <f>Table1[[#This Row],[FP]]/Table1[[#This Row],[NFL.Games]]</f>
         <v>16.872</v>
       </c>
-      <c r="Z2" s="15">
+      <c r="Z2" s="13">
         <f>Table1[[#This Row],[FP]]/Table1[[#This Row],[Snaps]]</f>
         <v>0.23796897038081805</v>
       </c>
@@ -1464,19 +1462,19 @@
       </c>
       <c r="S3" s="4">
         <f ca="1">(TODAY()-R3)/365-1</f>
-        <v>23.134246575342466</v>
-      </c>
-      <c r="T3" s="11">
+        <v>25.17808219178082</v>
+      </c>
+      <c r="T3" s="10">
         <f>6*12</f>
         <v>72</v>
       </c>
-      <c r="U3" s="11">
+      <c r="U3" s="10">
         <v>217</v>
       </c>
-      <c r="V3" s="11">
+      <c r="V3" s="10">
         <v>9</v>
       </c>
-      <c r="W3" s="11">
+      <c r="W3" s="10">
         <v>571</v>
       </c>
       <c r="X3" s="4">
@@ -1486,7 +1484,7 @@
         <f>Table1[[#This Row],[FP]]/Table1[[#This Row],[NFL.Games]]</f>
         <v>14.606666666666667</v>
       </c>
-      <c r="Z3" s="15">
+      <c r="Z3" s="13">
         <f>Table1[[#This Row],[FP]]/Table1[[#This Row],[Snaps]]</f>
         <v>0.2302276707530648</v>
       </c>
@@ -1549,19 +1547,19 @@
       </c>
       <c r="S4" s="4">
         <f ca="1">(TODAY()-R4)/365-1</f>
-        <v>23.112328767123287</v>
-      </c>
-      <c r="T4" s="11">
+        <v>25.156164383561645</v>
+      </c>
+      <c r="T4" s="10">
         <f>6*12+6</f>
         <v>78</v>
       </c>
-      <c r="U4" s="11">
+      <c r="U4" s="10">
         <v>236</v>
       </c>
-      <c r="V4" s="11">
+      <c r="V4" s="10">
         <v>15</v>
       </c>
-      <c r="W4" s="11">
+      <c r="W4" s="10">
         <v>1097</v>
       </c>
       <c r="X4" s="4">
@@ -1571,7 +1569,7 @@
         <f>Table1[[#This Row],[FP]]/Table1[[#This Row],[NFL.Games]]</f>
         <v>21.789333333333332</v>
       </c>
-      <c r="Z4" s="15">
+      <c r="Z4" s="13">
         <f>Table1[[#This Row],[FP]]/Table1[[#This Row],[Snaps]]</f>
         <v>0.29793983591613488</v>
       </c>
@@ -1634,19 +1632,19 @@
       </c>
       <c r="S5" s="4">
         <f ca="1">(TODAY()-R5)/365-1</f>
-        <v>22.701369863013699</v>
-      </c>
-      <c r="T5" s="11">
+        <v>24.745205479452054</v>
+      </c>
+      <c r="T5" s="10">
         <f>6*12+1</f>
         <v>73</v>
       </c>
-      <c r="U5" s="11">
+      <c r="U5" s="10">
         <v>223</v>
       </c>
-      <c r="V5" s="11">
+      <c r="V5" s="10">
         <v>4</v>
       </c>
-      <c r="W5" s="11">
+      <c r="W5" s="10">
         <v>334</v>
       </c>
       <c r="X5" s="4">
@@ -1656,15 +1654,13 @@
         <f>Table1[[#This Row],[FP]]/Table1[[#This Row],[NFL.Games]]</f>
         <v>25.484999999999999</v>
       </c>
-      <c r="Z5" s="15">
+      <c r="Z5" s="13">
         <f>Table1[[#This Row],[FP]]/Table1[[#This Row],[Snaps]]</f>
         <v>0.30520958083832334</v>
       </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="P9" s="7"/>
-      <c r="Q9" s="8"/>
-      <c r="R9" s="8"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Z5">
@@ -1688,97 +1684,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="13" t="s">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="L1" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="M1" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="N1" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="O1" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="P1" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="Q1" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="R1" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="S1" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="T1" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="U1" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="V1" s="13" t="s">
+      <c r="V1" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="W1" s="13" t="s">
+      <c r="W1" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="X1" s="13" t="s">
+      <c r="X1" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="Y1" s="13" t="s">
+      <c r="Y1" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="Z1" s="13" t="s">
+      <c r="Z1" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="AA1" s="13" t="s">
+      <c r="AA1" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="AB1" s="13" t="s">
+      <c r="AB1" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="AC1" s="13" t="s">
+      <c r="AC1" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="AD1" s="13" t="s">
+      <c r="AD1" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="AE1" s="13" t="s">
+      <c r="AE1" s="11" t="s">
         <v>126</v>
       </c>
     </row>
@@ -1822,31 +1818,31 @@
       <c r="M2">
         <v>1</v>
       </c>
-      <c r="N2" s="11">
+      <c r="N2" s="10">
         <f>215/494*100</f>
         <v>43.522267206477736</v>
       </c>
-      <c r="O2" s="11">
+      <c r="O2" s="10">
         <f>1414/2537*100</f>
         <v>55.735120220733151</v>
       </c>
-      <c r="P2" s="11">
+      <c r="P2" s="10">
         <f>55/426*100</f>
         <v>12.910798122065728</v>
       </c>
-      <c r="Q2" s="11">
+      <c r="Q2" s="10">
         <f>453/6024*100</f>
         <v>7.5199203187250996</v>
       </c>
-      <c r="R2" s="11">
+      <c r="R2" s="10">
         <f>1867/8561*100</f>
         <v>21.808199976638242</v>
       </c>
-      <c r="S2" s="11">
+      <c r="S2" s="10">
         <f>270/920*100</f>
         <v>29.347826086956523</v>
       </c>
-      <c r="T2" s="11">
+      <c r="T2" s="10">
         <f>1884/8654*100</f>
         <v>21.770279639473074</v>
       </c>
@@ -1861,19 +1857,19 @@
       </c>
       <c r="X2" s="4">
         <f t="shared" ref="X2:X12" ca="1" si="0">(TODAY()-W2)/365-1</f>
-        <v>22.024657534246575</v>
-      </c>
-      <c r="Y2" s="11">
+        <v>24.068493150684933</v>
+      </c>
+      <c r="Y2" s="10">
         <f>5*12+7</f>
         <v>67</v>
       </c>
-      <c r="Z2" s="11">
+      <c r="Z2" s="10">
         <v>207</v>
       </c>
-      <c r="AA2" s="11">
+      <c r="AA2" s="10">
         <v>13</v>
       </c>
-      <c r="AB2" s="11">
+      <c r="AB2" s="10">
         <v>542</v>
       </c>
       <c r="AC2" s="4">
@@ -1883,7 +1879,7 @@
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[NFL.Games]]</f>
         <v>12.153846153846153</v>
       </c>
-      <c r="AE2" s="15">
+      <c r="AE2" s="13">
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[Snaps]]</f>
         <v>0.29151291512915128</v>
       </c>
@@ -1928,31 +1924,31 @@
       <c r="M3">
         <v>1</v>
       </c>
-      <c r="N3" s="11">
+      <c r="N3" s="10">
         <f>196/505*100</f>
         <v>38.811881188118811</v>
       </c>
-      <c r="O3" s="11">
+      <c r="O3" s="10">
         <f>1218/2652*100</f>
         <v>45.927601809954751</v>
       </c>
-      <c r="P3" s="11">
+      <c r="P3" s="10">
         <f>24/255*100</f>
         <v>9.4117647058823533</v>
       </c>
-      <c r="Q3" s="11">
+      <c r="Q3" s="10">
         <f>216/3122*100</f>
         <v>6.9186418962203717</v>
       </c>
-      <c r="R3" s="11">
+      <c r="R3" s="10">
         <f>1434/5774*100</f>
         <v>24.835469345341185</v>
       </c>
-      <c r="S3" s="11">
+      <c r="S3" s="10">
         <f>220/760*100</f>
         <v>28.947368421052634</v>
       </c>
-      <c r="T3" s="11">
+      <c r="T3" s="10">
         <f>1442/5821*100</f>
         <v>24.772375880432914</v>
       </c>
@@ -1967,19 +1963,19 @@
       </c>
       <c r="X3" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>22.263013698630136</v>
-      </c>
-      <c r="Y3" s="11">
+        <v>24.306849315068494</v>
+      </c>
+      <c r="Y3" s="10">
         <f>5*12+9</f>
         <v>69</v>
       </c>
-      <c r="Z3" s="11">
+      <c r="Z3" s="10">
         <v>215</v>
       </c>
-      <c r="AA3" s="11">
+      <c r="AA3" s="10">
         <v>11</v>
       </c>
-      <c r="AB3" s="11">
+      <c r="AB3" s="10">
         <v>398</v>
       </c>
       <c r="AC3" s="4">
@@ -1989,7 +1985,7 @@
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[NFL.Games]]</f>
         <v>15.072727272727274</v>
       </c>
-      <c r="AE3" s="15">
+      <c r="AE3" s="13">
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[Snaps]]</f>
         <v>0.41658291457286434</v>
       </c>
@@ -2034,31 +2030,31 @@
       <c r="M4">
         <v>5</v>
       </c>
-      <c r="N4" s="11">
+      <c r="N4" s="10">
         <f>320/600*100</f>
         <v>53.333333333333336</v>
       </c>
-      <c r="O4" s="11">
+      <c r="O4" s="10">
         <f>2003/3278*100</f>
         <v>61.104331909701038</v>
       </c>
-      <c r="P4" s="11">
+      <c r="P4" s="10">
         <f>26/246*100</f>
         <v>10.569105691056912</v>
       </c>
-      <c r="Q4" s="11">
+      <c r="Q4" s="10">
         <f>252/2802*100</f>
         <v>8.9935760171306214</v>
       </c>
-      <c r="R4" s="11">
+      <c r="R4" s="10">
         <f>2255/6080*100</f>
         <v>37.088815789473685</v>
       </c>
-      <c r="S4" s="11">
+      <c r="S4" s="10">
         <f>346/846*100</f>
         <v>40.898345153664302</v>
       </c>
-      <c r="T4" s="11">
+      <c r="T4" s="10">
         <f>2281/6136*100</f>
         <v>37.174054758800523</v>
       </c>
@@ -2073,19 +2069,19 @@
       </c>
       <c r="X4" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>22.24931506849315</v>
-      </c>
-      <c r="Y4" s="11">
+        <v>24.293150684931508</v>
+      </c>
+      <c r="Y4" s="10">
         <f>5*12+10</f>
         <v>70</v>
       </c>
-      <c r="Z4" s="11">
+      <c r="Z4" s="10">
         <v>226</v>
       </c>
-      <c r="AA4" s="11">
+      <c r="AA4" s="10">
         <v>12</v>
       </c>
-      <c r="AB4" s="11">
+      <c r="AB4" s="10">
         <v>511</v>
       </c>
       <c r="AC4" s="4">
@@ -2095,7 +2091,7 @@
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[NFL.Games]]</f>
         <v>19.566666666666666</v>
       </c>
-      <c r="AE4" s="15">
+      <c r="AE4" s="13">
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[Snaps]]</f>
         <v>0.45949119373776909</v>
       </c>
@@ -2140,31 +2136,31 @@
       <c r="M5">
         <v>1</v>
       </c>
-      <c r="N5" s="11">
+      <c r="N5" s="10">
         <f>231/468*100</f>
         <v>49.358974358974365</v>
       </c>
-      <c r="O5" s="11">
+      <c r="O5" s="10">
         <f>1144/1898*100</f>
         <v>60.273972602739725</v>
       </c>
-      <c r="P5" s="11">
+      <c r="P5" s="10">
         <f>30/279*100</f>
         <v>10.75268817204301</v>
       </c>
-      <c r="Q5" s="11">
+      <c r="Q5" s="10">
         <f>225/3479*100</f>
         <v>6.4673756826674325</v>
       </c>
-      <c r="R5" s="11">
+      <c r="R5" s="10">
         <f>1369/5377*100</f>
         <v>25.460293844151018</v>
       </c>
-      <c r="S5" s="11">
+      <c r="S5" s="10">
         <f>261/747*100</f>
         <v>34.939759036144579</v>
       </c>
-      <c r="T5" s="11">
+      <c r="T5" s="10">
         <f>1387/5425*100</f>
         <v>25.566820276497698</v>
       </c>
@@ -2179,19 +2175,19 @@
       </c>
       <c r="X5" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>21.827397260273973</v>
-      </c>
-      <c r="Y5" s="11">
+        <v>23.87123287671233</v>
+      </c>
+      <c r="Y5" s="10">
         <f>5*12+10</f>
         <v>70</v>
       </c>
-      <c r="Z5" s="11">
+      <c r="Z5" s="10">
         <v>217</v>
       </c>
-      <c r="AA5" s="11">
+      <c r="AA5" s="10">
         <v>4</v>
       </c>
-      <c r="AB5" s="11">
+      <c r="AB5" s="10">
         <v>297</v>
       </c>
       <c r="AC5" s="4">
@@ -2201,7 +2197,7 @@
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[NFL.Games]]</f>
         <v>24.074999999999999</v>
       </c>
-      <c r="AE5" s="15">
+      <c r="AE5" s="13">
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[Snaps]]</f>
         <v>0.32424242424242422</v>
       </c>
@@ -2246,31 +2242,31 @@
       <c r="M6">
         <v>2</v>
       </c>
-      <c r="N6" s="11">
+      <c r="N6" s="10">
         <f>301/647*100</f>
         <v>46.522411128284389</v>
       </c>
-      <c r="O6" s="11">
+      <c r="O6" s="10">
         <f>2003/3770*100</f>
         <v>53.129973474801062</v>
       </c>
-      <c r="P6" s="11">
+      <c r="P6" s="10">
         <f>23/271*100</f>
         <v>8.4870848708487081</v>
       </c>
-      <c r="Q6" s="11">
+      <c r="Q6" s="10">
         <f>247/3684*100</f>
         <v>6.7046688382193267</v>
       </c>
-      <c r="R6" s="11">
+      <c r="R6" s="10">
         <f>(2003+247)/(3770+3684)*100</f>
         <v>30.185135497719344</v>
       </c>
-      <c r="S6" s="11">
+      <c r="S6" s="10">
         <f>(23+301)/(647+271)*100</f>
         <v>35.294117647058826</v>
       </c>
-      <c r="T6" s="11">
+      <c r="T6" s="10">
         <f>(247+2+2003+21)/(3770+39+3684+48)*100</f>
         <v>30.141890995889138</v>
       </c>
@@ -2285,19 +2281,19 @@
       </c>
       <c r="X6" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>22.339726027397262</v>
-      </c>
-      <c r="Y6" s="11">
+        <v>24.383561643835616</v>
+      </c>
+      <c r="Y6" s="10">
         <f>5*12+10</f>
         <v>70</v>
       </c>
-      <c r="Z6" s="11">
+      <c r="Z6" s="10">
         <v>212</v>
       </c>
-      <c r="AA6" s="11">
+      <c r="AA6" s="10">
         <v>13</v>
       </c>
-      <c r="AB6" s="11">
+      <c r="AB6" s="10">
         <v>456</v>
       </c>
       <c r="AC6" s="4">
@@ -2307,7 +2303,7 @@
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[NFL.Games]]</f>
         <v>12.115384615384615</v>
       </c>
-      <c r="AE6" s="15">
+      <c r="AE6" s="13">
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[Snaps]]</f>
         <v>0.34539473684210525</v>
       </c>
@@ -2352,31 +2348,31 @@
       <c r="M7">
         <v>8</v>
       </c>
-      <c r="N7" s="11">
+      <c r="N7" s="10">
         <f>33/536*100</f>
         <v>6.1567164179104479</v>
       </c>
-      <c r="O7" s="11">
+      <c r="O7" s="10">
         <f>369/2703*100</f>
         <v>13.651498335183129</v>
       </c>
-      <c r="P7" s="11">
+      <c r="P7" s="10">
         <f>38/281*100</f>
         <v>13.523131672597867</v>
       </c>
-      <c r="Q7" s="11">
+      <c r="Q7" s="10">
         <f>735/4177*100</f>
         <v>17.596361024658847</v>
       </c>
-      <c r="R7" s="11">
+      <c r="R7" s="10">
         <f>(735+369)/(2703+4177)*100</f>
         <v>16.046511627906977</v>
       </c>
-      <c r="S7" s="11">
+      <c r="S7" s="10">
         <f>(38+33)/(536+281)*100</f>
         <v>8.6903304773561807</v>
       </c>
-      <c r="T7" s="11">
+      <c r="T7" s="10">
         <f>(369+4+8+735)/(2703+32+4177+33)*100</f>
         <v>16.069114470842333</v>
       </c>
@@ -2391,19 +2387,19 @@
       </c>
       <c r="X7" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>22.824657534246576</v>
-      </c>
-      <c r="Y7" s="11">
+        <v>24.86849315068493</v>
+      </c>
+      <c r="Y7" s="10">
         <f>6*12</f>
         <v>72</v>
       </c>
-      <c r="Z7" s="11">
+      <c r="Z7" s="10">
         <v>228</v>
       </c>
-      <c r="AA7" s="11">
+      <c r="AA7" s="10">
         <v>11</v>
       </c>
-      <c r="AB7" s="11">
+      <c r="AB7" s="10">
         <v>405</v>
       </c>
       <c r="AC7" s="4">
@@ -2413,7 +2409,7 @@
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[NFL.Games]]</f>
         <v>16.745454545454546</v>
       </c>
-      <c r="AE7" s="15">
+      <c r="AE7" s="13">
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[Snaps]]</f>
         <v>0.45481481481481478</v>
       </c>
@@ -2458,31 +2454,31 @@
       <c r="M8">
         <v>1</v>
       </c>
-      <c r="N8" s="11">
+      <c r="N8" s="10">
         <f>198/357*100</f>
         <v>55.462184873949582</v>
       </c>
-      <c r="O8" s="11">
+      <c r="O8" s="10">
         <f>1028/1526*100</f>
         <v>67.365661861074713</v>
       </c>
-      <c r="P8" s="11">
+      <c r="P8" s="10">
         <f>28/202*100</f>
         <v>13.861386138613863</v>
       </c>
-      <c r="Q8" s="11">
+      <c r="Q8" s="10">
         <f>270/2064*100</f>
         <v>13.08139534883721</v>
       </c>
-      <c r="R8" s="11">
+      <c r="R8" s="10">
         <f>(270+1028)/(1526+2064)*100</f>
         <v>36.155988857938723</v>
       </c>
-      <c r="S8" s="11">
+      <c r="S8" s="10">
         <f>(28+198)/(357+202)*100</f>
         <v>40.429338103756706</v>
       </c>
-      <c r="T8" s="11">
+      <c r="T8" s="10">
         <f>(270+1+9+1028)/(1526+11+2064+10)*100</f>
         <v>36.222653004707837</v>
       </c>
@@ -2497,19 +2493,19 @@
       </c>
       <c r="X8" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>23.961643835616439</v>
-      </c>
-      <c r="Y8" s="11">
+        <v>26.005479452054793</v>
+      </c>
+      <c r="Y8" s="10">
         <f>5*12+10</f>
         <v>70</v>
       </c>
-      <c r="Z8" s="11">
+      <c r="Z8" s="10">
         <v>214</v>
       </c>
-      <c r="AA8" s="11">
+      <c r="AA8" s="10">
         <v>1</v>
       </c>
-      <c r="AB8" s="11">
+      <c r="AB8" s="10">
         <v>99</v>
       </c>
       <c r="AC8" s="4">
@@ -2519,7 +2515,7 @@
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[NFL.Games]]</f>
         <v>20.8</v>
       </c>
-      <c r="AE8" s="15">
+      <c r="AE8" s="13">
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[Snaps]]</f>
         <v>0.21010101010101012</v>
       </c>
@@ -2564,31 +2560,31 @@
       <c r="M9">
         <v>2</v>
       </c>
-      <c r="N9" s="11">
+      <c r="N9" s="10">
         <f>235/583*100</f>
         <v>40.308747855917666</v>
       </c>
-      <c r="O9" s="11">
+      <c r="O9" s="10">
         <f>1416/2832*100</f>
         <v>50</v>
       </c>
-      <c r="P9" s="11">
+      <c r="P9" s="10">
         <f>28/233*100</f>
         <v>12.017167381974248</v>
       </c>
-      <c r="Q9" s="11">
+      <c r="Q9" s="10">
         <f>388/3187*100</f>
         <v>12.174458738625667</v>
       </c>
-      <c r="R9" s="11">
+      <c r="R9" s="10">
         <f>(388+1416)/(2832+3187)*100</f>
         <v>29.971756105665392</v>
       </c>
-      <c r="S9" s="11">
+      <c r="S9" s="10">
         <f>(28+235)/(583+233)*100</f>
         <v>32.230392156862749</v>
       </c>
-      <c r="T9" s="11">
+      <c r="T9" s="10">
         <f>(1416+15+388+2)/(3187+20+34+2832)*100</f>
         <v>29.985180306273669</v>
       </c>
@@ -2603,19 +2599,19 @@
       </c>
       <c r="X9" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>23.342465753424658</v>
-      </c>
-      <c r="Y9" s="11">
+        <v>25.386301369863013</v>
+      </c>
+      <c r="Y9" s="10">
         <f>5*12+9</f>
         <v>69</v>
       </c>
-      <c r="Z9" s="11">
+      <c r="Z9" s="10">
         <v>205</v>
       </c>
-      <c r="AA9" s="11">
+      <c r="AA9" s="10">
         <v>10</v>
       </c>
-      <c r="AB9" s="11">
+      <c r="AB9" s="10">
         <v>403</v>
       </c>
       <c r="AC9" s="4">
@@ -2625,7 +2621,7 @@
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[NFL.Games]]</f>
         <v>9.4599999999999991</v>
       </c>
-      <c r="AE9" s="15">
+      <c r="AE9" s="13">
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[Snaps]]</f>
         <v>0.23473945409429278</v>
       </c>
@@ -2670,31 +2666,31 @@
       <c r="M10">
         <v>1</v>
       </c>
-      <c r="N10" s="11">
+      <c r="N10" s="10">
         <f>229/484*100</f>
         <v>47.314049586776861</v>
       </c>
-      <c r="O10" s="11">
+      <c r="O10" s="10">
         <f>1060/1826*100</f>
         <v>58.050383351588174</v>
       </c>
-      <c r="P10" s="11">
+      <c r="P10" s="10">
         <f>11/260*100</f>
         <v>4.2307692307692308</v>
       </c>
-      <c r="Q10" s="11">
+      <c r="Q10" s="10">
         <f>71/3066*100</f>
         <v>2.3157208088714936</v>
       </c>
-      <c r="R10" s="11">
+      <c r="R10" s="10">
         <f>(71+1060)/(1826+3066)*100</f>
         <v>23.119378577269011</v>
       </c>
-      <c r="S10" s="11">
+      <c r="S10" s="10">
         <f>(11+229)/(484+260)*100</f>
         <v>32.258064516129032</v>
       </c>
-      <c r="T10" s="11">
+      <c r="T10" s="10">
         <f>(71+1+12+1060)/(1826+18+3066+22)*100</f>
         <v>23.195458231954582</v>
       </c>
@@ -2709,19 +2705,19 @@
       </c>
       <c r="X10" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>23.413698630136988</v>
-      </c>
-      <c r="Y10" s="11">
+        <v>25.457534246575342</v>
+      </c>
+      <c r="Y10" s="10">
         <f>5*12+11</f>
         <v>71</v>
       </c>
-      <c r="Z10" s="11">
+      <c r="Z10" s="10">
         <v>212</v>
       </c>
-      <c r="AA10" s="11">
+      <c r="AA10" s="10">
         <v>5</v>
       </c>
-      <c r="AB10" s="11">
+      <c r="AB10" s="10">
         <v>297</v>
       </c>
       <c r="AC10" s="4">
@@ -2731,7 +2727,7 @@
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[NFL.Games]]</f>
         <v>13.940000000000001</v>
       </c>
-      <c r="AE10" s="15">
+      <c r="AE10" s="13">
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[Snaps]]</f>
         <v>0.23468013468013468</v>
       </c>
@@ -2776,31 +2772,31 @@
       <c r="M11">
         <v>5</v>
       </c>
-      <c r="N11" s="11">
+      <c r="N11" s="10">
         <f>132/392*100</f>
         <v>33.673469387755098</v>
       </c>
-      <c r="O11" s="11">
+      <c r="O11" s="10">
         <f>676/1694*100</f>
         <v>39.905548996458087</v>
       </c>
-      <c r="P11" s="11">
+      <c r="P11" s="10">
         <f>40/317*100</f>
         <v>12.618296529968454</v>
       </c>
-      <c r="Q11" s="11">
+      <c r="Q11" s="10">
         <f>262/3910*100</f>
         <v>6.7007672634271103</v>
       </c>
-      <c r="R11" s="11">
+      <c r="R11" s="10">
         <f>(262+676)/(1694+3910)*100</f>
         <v>16.73804425410421</v>
       </c>
-      <c r="S11" s="11">
+      <c r="S11" s="10">
         <f>(40+132)/(392+317)*100</f>
         <v>24.259520451339917</v>
       </c>
-      <c r="T11" s="11">
+      <c r="T11" s="10">
         <f>(262+5+6+676)/(1694+21+3910+33)*100</f>
         <v>16.772711205372921</v>
       </c>
@@ -2815,19 +2811,19 @@
       </c>
       <c r="X11" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>23.219178082191782</v>
-      </c>
-      <c r="Y11" s="11">
+        <v>25.263013698630136</v>
+      </c>
+      <c r="Y11" s="10">
         <f>5*12+11</f>
         <v>71</v>
       </c>
-      <c r="Z11" s="11">
+      <c r="Z11" s="10">
         <v>216</v>
       </c>
-      <c r="AA11" s="11">
+      <c r="AA11" s="10">
         <v>4</v>
       </c>
-      <c r="AB11" s="11">
+      <c r="AB11" s="10">
         <v>200</v>
       </c>
       <c r="AC11" s="4">
@@ -2837,7 +2833,7 @@
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[NFL.Games]]</f>
         <v>11.75</v>
       </c>
-      <c r="AE11" s="15">
+      <c r="AE11" s="13">
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[Snaps]]</f>
         <v>0.23499999999999999</v>
       </c>
@@ -2882,31 +2878,31 @@
       <c r="M12">
         <v>0</v>
       </c>
-      <c r="N12" s="11">
+      <c r="N12" s="10">
         <f>364/645*100</f>
         <v>56.434108527131791</v>
       </c>
-      <c r="O12" s="11">
+      <c r="O12" s="10">
         <f>1899/2733*100</f>
         <v>69.484083424807906</v>
       </c>
-      <c r="P12" s="11">
+      <c r="P12" s="10">
         <f>16/132*100</f>
         <v>12.121212121212121</v>
       </c>
-      <c r="Q12" s="11">
+      <c r="Q12" s="10">
         <f>80/1767*100</f>
         <v>4.5274476513865309</v>
       </c>
-      <c r="R12" s="11">
+      <c r="R12" s="10">
         <f>(80+1899)/(2733+1767)*100</f>
         <v>43.977777777777774</v>
       </c>
-      <c r="S12" s="11">
+      <c r="S12" s="10">
         <f>(16+364)/(645+132)*100</f>
         <v>48.906048906048902</v>
       </c>
-      <c r="T12" s="11">
+      <c r="T12" s="10">
         <f>(80+1899+18)/(2733+24+1767+10)*100</f>
         <v>44.044993383325981</v>
       </c>
@@ -2921,19 +2917,19 @@
       </c>
       <c r="X12" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>22.695890410958903</v>
-      </c>
-      <c r="Y12" s="11">
+        <v>24.739726027397261</v>
+      </c>
+      <c r="Y12" s="10">
         <f>5*12+9</f>
         <v>69</v>
       </c>
-      <c r="Z12" s="11">
+      <c r="Z12" s="10">
         <v>219</v>
       </c>
-      <c r="AA12" s="11">
+      <c r="AA12" s="10">
         <v>14</v>
       </c>
-      <c r="AB12" s="11">
+      <c r="AB12" s="10">
         <v>641</v>
       </c>
       <c r="AC12" s="4">
@@ -2943,7 +2939,7 @@
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[NFL.Games]]</f>
         <v>15.992857142857144</v>
       </c>
-      <c r="AE12" s="15">
+      <c r="AE12" s="13">
         <f>Table2[[#This Row],[FP]]/Table2[[#This Row],[Snaps]]</f>
         <v>0.34929797191887674</v>
       </c>
@@ -3005,7 +3001,7 @@
   <cols>
     <col min="1" max="1" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="18" width="0" hidden="1" customWidth="1"/>
+    <col min="5" max="18" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3096,665 +3092,662 @@
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>46</v>
+        <v>121</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>61</v>
+        <v>14</v>
       </c>
       <c r="C2">
-        <v>92</v>
+        <v>12</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="E2" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F2">
-        <v>106</v>
+        <v>40</v>
       </c>
       <c r="G2">
-        <v>1386</v>
+        <v>746</v>
       </c>
       <c r="H2" s="4">
-        <v>13.08</v>
+        <v>18.649999999999999</v>
       </c>
       <c r="I2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K2">
-        <v>24</v>
+        <v>75</v>
       </c>
       <c r="L2" s="4">
-        <v>2.4</v>
+        <v>37.5</v>
       </c>
       <c r="M2">
         <v>1</v>
       </c>
-      <c r="N2" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="O2" s="12">
-        <f>106/306*100</f>
-        <v>34.640522875816991</v>
-      </c>
-      <c r="P2" s="12">
-        <f>1386/3761*100</f>
-        <v>36.851901090135605</v>
-      </c>
-      <c r="Q2" s="12">
-        <f>9/32*100</f>
-        <v>28.125</v>
-      </c>
-      <c r="R2" s="12">
-        <f>(1386+9)/(3761+32)*100</f>
-        <v>36.778275771157389</v>
-      </c>
-      <c r="S2" s="16">
-        <v>20.879000000000001</v>
-      </c>
-      <c r="T2" s="9">
-        <v>35685</v>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2" s="10">
+        <f>40/287*100</f>
+        <v>13.937282229965156</v>
+      </c>
+      <c r="P2" s="10">
+        <f>746/4449*100</f>
+        <v>16.767812991683524</v>
+      </c>
+      <c r="Q2" s="10">
+        <f>7/49*100</f>
+        <v>14.285714285714285</v>
+      </c>
+      <c r="R2" s="10">
+        <f>(746+7)/(4449+49)*100</f>
+        <v>16.740773677189864</v>
+      </c>
+      <c r="S2" s="4">
+        <v>47.41</v>
+      </c>
+      <c r="T2" s="7">
+        <v>36184</v>
       </c>
       <c r="U2" s="5">
-        <f t="shared" ref="U2:U21" ca="1" si="0">((TODAY()-T2)/365)-1</f>
-        <v>23.602739726027398</v>
-      </c>
-      <c r="V2" s="11">
+        <f ca="1">((TODAY()-T2)/365)-1</f>
+        <v>24.279452054794522</v>
+      </c>
+      <c r="V2" s="10">
+        <f>6*12</f>
+        <v>72</v>
+      </c>
+      <c r="W2" s="10">
+        <v>190</v>
+      </c>
+      <c r="X2" s="10">
+        <v>13</v>
+      </c>
+      <c r="Y2" s="10">
+        <v>581</v>
+      </c>
+      <c r="Z2" s="4">
+        <v>71.099999999999994</v>
+      </c>
+      <c r="AA2" s="4">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
+        <v>5.4692307692307685</v>
+      </c>
+      <c r="AB2" s="13">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
+        <v>0.12237521514629947</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3">
+        <v>15</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E3" s="1">
+        <v>13</v>
+      </c>
+      <c r="F3">
+        <v>77</v>
+      </c>
+      <c r="G3">
+        <v>1163</v>
+      </c>
+      <c r="H3" s="4">
+        <v>15.1</v>
+      </c>
+      <c r="I3">
+        <v>10</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3" s="4">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3" s="10">
+        <f>77/287*100</f>
+        <v>26.829268292682929</v>
+      </c>
+      <c r="P3" s="10">
+        <f>1163/4449*100</f>
+        <v>26.140705776579004</v>
+      </c>
+      <c r="Q3" s="10">
+        <f>10/49*100</f>
+        <v>20.408163265306122</v>
+      </c>
+      <c r="R3" s="10">
+        <f>(1163+10)/(4449+49)*100</f>
+        <v>26.078257003112494</v>
+      </c>
+      <c r="S3" s="4">
+        <f>44/262*100</f>
+        <v>16.793893129770993</v>
+      </c>
+      <c r="T3" s="7">
+        <v>36274</v>
+      </c>
+      <c r="U3" s="5">
+        <f ca="1">((TODAY()-T3)/365)-1</f>
+        <v>24.032876712328768</v>
+      </c>
+      <c r="V3" s="10">
+        <f>6*12+1</f>
+        <v>73</v>
+      </c>
+      <c r="W3" s="10">
+        <v>193</v>
+      </c>
+      <c r="X3" s="10">
+        <v>16</v>
+      </c>
+      <c r="Y3" s="10">
+        <v>806</v>
+      </c>
+      <c r="Z3" s="4">
+        <v>129.6</v>
+      </c>
+      <c r="AA3" s="4">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
+        <v>8.1</v>
+      </c>
+      <c r="AB3" s="13">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
+        <v>0.1607940446650124</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>17</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E4" s="1">
+        <v>13</v>
+      </c>
+      <c r="F4">
+        <v>62</v>
+      </c>
+      <c r="G4">
+        <v>1327</v>
+      </c>
+      <c r="H4" s="4">
+        <v>21.4</v>
+      </c>
+      <c r="I4">
+        <v>14</v>
+      </c>
+      <c r="J4">
+        <v>9</v>
+      </c>
+      <c r="K4">
+        <v>20</v>
+      </c>
+      <c r="L4" s="4">
+        <v>2.2200000000000002</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+      <c r="N4">
+        <v>2</v>
+      </c>
+      <c r="O4" s="10">
+        <f>62/262*100</f>
+        <v>23.664122137404579</v>
+      </c>
+      <c r="P4" s="10">
+        <f>1327/4164*100</f>
+        <v>31.86839577329491</v>
+      </c>
+      <c r="Q4" s="10">
+        <f>14/36*100</f>
+        <v>38.888888888888893</v>
+      </c>
+      <c r="R4" s="10">
+        <f>(1327+14)/(4164+36)*100</f>
+        <v>31.928571428571427</v>
+      </c>
+      <c r="S4" s="4">
+        <v>32.770000000000003</v>
+      </c>
+      <c r="T4" s="7">
+        <v>36258</v>
+      </c>
+      <c r="U4" s="5">
+        <f ca="1">((TODAY()-T4)/365)-1</f>
+        <v>24.076712328767123</v>
+      </c>
+      <c r="V4" s="10">
+        <f>6*12+2</f>
+        <v>74</v>
+      </c>
+      <c r="W4" s="10">
+        <v>189</v>
+      </c>
+      <c r="X4" s="10">
+        <v>16</v>
+      </c>
+      <c r="Y4" s="10">
+        <v>731</v>
+      </c>
+      <c r="Z4" s="4">
+        <v>179.7</v>
+      </c>
+      <c r="AA4" s="4">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
+        <v>11.231249999999999</v>
+      </c>
+      <c r="AB4" s="13">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
+        <v>0.24582763337893296</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5">
+        <v>21</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E5" s="1">
+        <v>12</v>
+      </c>
+      <c r="F5">
+        <v>43</v>
+      </c>
+      <c r="G5">
+        <v>611</v>
+      </c>
+      <c r="H5" s="4">
+        <v>14.21</v>
+      </c>
+      <c r="I5">
+        <v>5</v>
+      </c>
+      <c r="J5">
+        <v>14</v>
+      </c>
+      <c r="K5">
+        <v>89</v>
+      </c>
+      <c r="L5" s="4">
+        <v>6.36</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>6</v>
+      </c>
+      <c r="O5" s="10">
+        <f>43/211*100</f>
+        <v>20.379146919431278</v>
+      </c>
+      <c r="P5" s="10">
+        <f>611/2444*100</f>
+        <v>25</v>
+      </c>
+      <c r="Q5" s="10">
+        <f>5/15*100</f>
+        <v>33.333333333333329</v>
+      </c>
+      <c r="R5" s="10">
+        <f>(5+611)/(2444+15)*100</f>
+        <v>25.050833672224481</v>
+      </c>
+      <c r="S5" s="4">
+        <v>42.23</v>
+      </c>
+      <c r="T5" s="7">
+        <v>36161</v>
+      </c>
+      <c r="U5" s="5">
+        <f ca="1">((TODAY()-T5)/365)-1</f>
+        <v>24.342465753424658</v>
+      </c>
+      <c r="V5" s="10">
         <f>5*12+11</f>
         <v>71</v>
       </c>
-      <c r="W2" s="11">
-        <v>210</v>
-      </c>
-      <c r="X2" s="11">
+      <c r="W5" s="10">
+        <v>197</v>
+      </c>
+      <c r="X5" s="10">
+        <v>10</v>
+      </c>
+      <c r="Y5" s="10">
+        <v>511</v>
+      </c>
+      <c r="Z5" s="4">
+        <v>70.7</v>
+      </c>
+      <c r="AA5" s="4">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
+        <v>7.07</v>
+      </c>
+      <c r="AB5" s="13">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
+        <v>0.13835616438356166</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>22</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E6" s="1">
+        <v>15</v>
+      </c>
+      <c r="F6">
+        <v>111</v>
+      </c>
+      <c r="G6">
+        <v>1540</v>
+      </c>
+      <c r="H6" s="4">
+        <v>13.87</v>
+      </c>
+      <c r="I6">
+        <v>18</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6" s="10">
+        <f>111/426*100</f>
+        <v>26.056338028169012</v>
+      </c>
+      <c r="P6" s="10">
+        <f>1540/6024*100</f>
+        <v>25.564409030544489</v>
+      </c>
+      <c r="Q6" s="10">
+        <f>18/61*100</f>
+        <v>29.508196721311474</v>
+      </c>
+      <c r="R6" s="10">
+        <f>(18+1540)/(6024+61)*100</f>
+        <v>25.603944124897289</v>
+      </c>
+      <c r="S6" s="4">
+        <v>52.63</v>
+      </c>
+      <c r="T6" s="7">
+        <v>36176</v>
+      </c>
+      <c r="U6" s="5">
+        <f ca="1">((TODAY()-T6)/365)-1</f>
+        <v>24.301369863013697</v>
+      </c>
+      <c r="V6" s="10">
+        <f>6*12+1</f>
+        <v>73</v>
+      </c>
+      <c r="W6" s="10">
+        <v>202</v>
+      </c>
+      <c r="X6" s="10">
+        <v>16</v>
+      </c>
+      <c r="Y6" s="10">
+        <v>886</v>
+      </c>
+      <c r="Z6" s="4">
+        <v>229.2</v>
+      </c>
+      <c r="AA6" s="4">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
+        <v>14.324999999999999</v>
+      </c>
+      <c r="AB6" s="13">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
+        <v>0.2586907449209932</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7">
+        <v>25</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="1">
+        <v>12</v>
+      </c>
+      <c r="F7">
+        <v>65</v>
+      </c>
+      <c r="G7">
+        <v>1192</v>
+      </c>
+      <c r="H7" s="4">
+        <v>18.34</v>
+      </c>
+      <c r="I7">
+        <v>8</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7">
         <v>6</v>
       </c>
-      <c r="Y2" s="11">
-        <v>347</v>
-      </c>
-      <c r="Z2" s="4">
-        <v>43.1</v>
-      </c>
-      <c r="AA2" s="4">
+      <c r="L7" s="4">
+        <v>6</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>1</v>
+      </c>
+      <c r="O7" s="10">
+        <f>65/233*100</f>
+        <v>27.896995708154503</v>
+      </c>
+      <c r="P7" s="10">
+        <f>1192/3235*100</f>
+        <v>36.84698608964451</v>
+      </c>
+      <c r="Q7" s="10">
+        <f>8/21*100</f>
+        <v>38.095238095238095</v>
+      </c>
+      <c r="R7" s="10">
+        <f>(8+1192)/(3235+21)*100</f>
+        <v>36.855036855036857</v>
+      </c>
+      <c r="S7" s="4">
+        <v>48.927</v>
+      </c>
+      <c r="T7" s="7">
+        <v>35871</v>
+      </c>
+      <c r="U7" s="5">
+        <f ca="1">((TODAY()-T7)/365)-1</f>
+        <v>25.136986301369863</v>
+      </c>
+      <c r="V7" s="10">
+        <f>6*12</f>
+        <v>72</v>
+      </c>
+      <c r="W7" s="10">
+        <v>200</v>
+      </c>
+      <c r="X7" s="10">
+        <v>12</v>
+      </c>
+      <c r="Y7" s="10">
+        <v>728</v>
+      </c>
+      <c r="Z7" s="4">
+        <v>154.5</v>
+      </c>
+      <c r="AA7" s="4">
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>7.1833333333333336</v>
-      </c>
-      <c r="AB2" s="15">
+        <v>12.875</v>
+      </c>
+      <c r="AB7" s="13">
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.12420749279538905</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C3">
-        <v>128</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E3" s="1">
-        <v>12</v>
-      </c>
-      <c r="F3">
-        <v>72</v>
-      </c>
-      <c r="G3">
-        <v>1241</v>
-      </c>
-      <c r="H3" s="4">
-        <v>17.239999999999998</v>
-      </c>
-      <c r="I3">
-        <v>12</v>
-      </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-      <c r="L3" s="4">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="N3">
-        <v>0</v>
-      </c>
-      <c r="O3" s="12">
-        <f>72/271*100</f>
-        <v>26.568265682656829</v>
-      </c>
-      <c r="P3" s="12">
-        <f>1241/4117*100</f>
-        <v>30.143308234151078</v>
-      </c>
-      <c r="Q3" s="12">
-        <f>12/36*100</f>
-        <v>33.333333333333329</v>
-      </c>
-      <c r="R3" s="12">
-        <f>(1241+12)/(4117+36)*100</f>
-        <v>30.170960751264147</v>
-      </c>
-      <c r="S3" s="4">
-        <v>11.18</v>
-      </c>
-      <c r="T3" s="7">
-        <v>36251</v>
-      </c>
-      <c r="U3" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>22.052054794520547</v>
-      </c>
-      <c r="V3" s="11">
-        <f>6*12+2</f>
-        <v>74</v>
-      </c>
-      <c r="W3" s="11">
-        <v>210</v>
-      </c>
-      <c r="X3" s="11">
+        <v>0.21222527472527472</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8">
+        <v>33</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E8" s="1">
         <v>15</v>
       </c>
-      <c r="Y3" s="11">
-        <v>797</v>
-      </c>
-      <c r="Z3" s="4">
-        <v>118.4</v>
-      </c>
-      <c r="AA3" s="4">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>7.8933333333333335</v>
-      </c>
-      <c r="AB3" s="15">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.14855708908406526</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="C4">
-        <v>173</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="E4" s="1">
+      <c r="F8">
+        <v>59</v>
+      </c>
+      <c r="G8">
+        <v>1167</v>
+      </c>
+      <c r="H8" s="4">
+        <v>19.78</v>
+      </c>
+      <c r="I8">
         <v>13</v>
       </c>
-      <c r="F4">
-        <v>48</v>
-      </c>
-      <c r="G4">
-        <v>713</v>
-      </c>
-      <c r="H4" s="4">
-        <f>Table3[[#This Row],[Rec.Yds]]/Table3[[#This Row],[Receptions]]</f>
-        <v>14.854166666666666</v>
-      </c>
-      <c r="I4">
-        <v>5</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4" s="4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>0</v>
-      </c>
-      <c r="O4" s="12">
-        <f>48/197*100</f>
-        <v>24.36548223350254</v>
-      </c>
-      <c r="P4" s="12">
-        <f>713/2679*100</f>
-        <v>26.614408361328856</v>
-      </c>
-      <c r="Q4" s="12">
-        <f>5/19*100</f>
-        <v>26.315789473684209</v>
-      </c>
-      <c r="R4" s="12">
-        <f>(5+713)/(19+2679)*100</f>
-        <v>26.612305411415864</v>
-      </c>
-      <c r="S4" s="4">
-        <f>48/350*100</f>
-        <v>13.714285714285715</v>
-      </c>
-      <c r="T4" s="7">
-        <v>35732</v>
-      </c>
-      <c r="U4" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>23.473972602739725</v>
-      </c>
-      <c r="V4" s="11">
-        <f>5*12+11</f>
-        <v>71</v>
-      </c>
-      <c r="W4" s="11">
-        <v>174</v>
-      </c>
-      <c r="X4" s="11">
-        <v>15</v>
-      </c>
-      <c r="Y4" s="11">
-        <v>781</v>
-      </c>
-      <c r="Z4" s="4">
-        <v>120.6</v>
-      </c>
-      <c r="AA4" s="4">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>8.0399999999999991</v>
-      </c>
-      <c r="AB4" s="15">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.15441741357234315</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C5">
-        <v>33</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="E5" s="1">
-        <v>15</v>
-      </c>
-      <c r="F5">
-        <v>59</v>
-      </c>
-      <c r="G5">
-        <v>1167</v>
-      </c>
-      <c r="H5" s="4">
-        <v>19.78</v>
-      </c>
-      <c r="I5">
-        <v>13</v>
-      </c>
-      <c r="J5">
+      <c r="J8">
         <v>1</v>
       </c>
-      <c r="K5">
+      <c r="K8">
         <v>36</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L8" s="4">
         <v>36</v>
       </c>
-      <c r="M5">
+      <c r="M8">
         <v>1</v>
       </c>
-      <c r="N5">
-        <v>0</v>
-      </c>
-      <c r="O5" s="11">
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8" s="10">
         <f>59/326*100</f>
         <v>18.098159509202453</v>
       </c>
-      <c r="P5" s="11">
+      <c r="P8" s="10">
         <f>1167/4325*100</f>
         <v>26.98265895953757</v>
       </c>
-      <c r="Q5" s="11">
+      <c r="Q8" s="10">
         <f>13/40*100</f>
         <v>32.5</v>
       </c>
-      <c r="R5" s="11">
+      <c r="R8" s="10">
         <f>(13+1167)/(4325+40)*100</f>
         <v>27.033218785796105</v>
       </c>
-      <c r="S5" s="4">
+      <c r="S8" s="4">
         <f>16/388*100</f>
         <v>4.1237113402061851</v>
       </c>
-      <c r="T5" s="7">
+      <c r="T8" s="7">
         <v>36178</v>
       </c>
-      <c r="U5" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>22.252054794520546</v>
-      </c>
-      <c r="V5" s="11">
+      <c r="U8" s="5">
+        <f ca="1">((TODAY()-T8)/365)-1</f>
+        <v>24.295890410958904</v>
+      </c>
+      <c r="V8" s="10">
         <f>6*12+4</f>
         <v>76</v>
       </c>
-      <c r="W5" s="11">
+      <c r="W8" s="10">
         <v>215</v>
       </c>
-      <c r="X5" s="11">
+      <c r="X8" s="10">
         <v>14</v>
       </c>
-      <c r="Y5" s="11">
+      <c r="Y8" s="10">
         <v>805</v>
       </c>
-      <c r="Z5" s="4">
+      <c r="Z8" s="4">
         <v>161.1</v>
       </c>
-      <c r="AA5" s="4">
+      <c r="AA8" s="4">
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
         <v>11.507142857142856</v>
       </c>
-      <c r="AB5" s="15">
+      <c r="AB8" s="13">
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
         <v>0.20012422360248447</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6">
-        <v>17</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="E6" s="1">
-        <v>13</v>
-      </c>
-      <c r="F6">
-        <v>62</v>
-      </c>
-      <c r="G6">
-        <v>1327</v>
-      </c>
-      <c r="H6" s="4">
-        <v>21.4</v>
-      </c>
-      <c r="I6">
-        <v>14</v>
-      </c>
-      <c r="J6">
-        <v>9</v>
-      </c>
-      <c r="K6">
-        <v>20</v>
-      </c>
-      <c r="L6" s="4">
-        <v>2.2200000000000002</v>
-      </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-      <c r="N6">
-        <v>2</v>
-      </c>
-      <c r="O6" s="11">
-        <f>62/262*100</f>
-        <v>23.664122137404579</v>
-      </c>
-      <c r="P6" s="11">
-        <f>1327/4164*100</f>
-        <v>31.86839577329491</v>
-      </c>
-      <c r="Q6" s="11">
-        <f>14/36*100</f>
-        <v>38.888888888888893</v>
-      </c>
-      <c r="R6" s="11">
-        <f>(1327+14)/(4164+36)*100</f>
-        <v>31.928571428571427</v>
-      </c>
-      <c r="S6" s="4">
-        <v>32.770000000000003</v>
-      </c>
-      <c r="T6" s="7">
-        <v>36258</v>
-      </c>
-      <c r="U6" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>22.032876712328768</v>
-      </c>
-      <c r="V6" s="11">
-        <f>6*12+2</f>
-        <v>74</v>
-      </c>
-      <c r="W6" s="11">
-        <v>189</v>
-      </c>
-      <c r="X6" s="11">
-        <v>16</v>
-      </c>
-      <c r="Y6" s="11">
-        <v>731</v>
-      </c>
-      <c r="Z6" s="4">
-        <v>179.7</v>
-      </c>
-      <c r="AA6" s="4">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>11.231249999999999</v>
-      </c>
-      <c r="AB6" s="15">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.24582763337893296</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7">
-        <v>15</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="E7" s="1">
-        <v>13</v>
-      </c>
-      <c r="F7">
-        <v>77</v>
-      </c>
-      <c r="G7">
-        <v>1163</v>
-      </c>
-      <c r="H7" s="4">
-        <v>15.1</v>
-      </c>
-      <c r="I7">
-        <v>10</v>
-      </c>
-      <c r="J7">
-        <v>1</v>
-      </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="L7" s="4">
-        <v>1</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7">
-        <v>0</v>
-      </c>
-      <c r="O7" s="11">
-        <f>77/287*100</f>
-        <v>26.829268292682929</v>
-      </c>
-      <c r="P7" s="11">
-        <f>1163/4449*100</f>
-        <v>26.140705776579004</v>
-      </c>
-      <c r="Q7" s="11">
-        <f>10/49*100</f>
-        <v>20.408163265306122</v>
-      </c>
-      <c r="R7" s="11">
-        <f>(1163+10)/(4449+49)*100</f>
-        <v>26.078257003112494</v>
-      </c>
-      <c r="S7" s="4">
-        <f>44/262*100</f>
-        <v>16.793893129770993</v>
-      </c>
-      <c r="T7" s="7">
-        <v>36274</v>
-      </c>
-      <c r="U7" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>21.989041095890411</v>
-      </c>
-      <c r="V7" s="11">
-        <f>6*12+1</f>
-        <v>73</v>
-      </c>
-      <c r="W7" s="11">
-        <v>193</v>
-      </c>
-      <c r="X7" s="11">
-        <v>16</v>
-      </c>
-      <c r="Y7" s="11">
-        <v>806</v>
-      </c>
-      <c r="Z7" s="4">
-        <v>129.6</v>
-      </c>
-      <c r="AA7" s="4">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>8.1</v>
-      </c>
-      <c r="AB7" s="15">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.1607940446650124</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8">
-        <v>46</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="E8" s="1">
-        <v>13</v>
-      </c>
-      <c r="F8">
-        <v>56</v>
-      </c>
-      <c r="G8">
-        <v>904</v>
-      </c>
-      <c r="H8" s="4">
-        <v>16.14</v>
-      </c>
-      <c r="I8">
-        <v>8</v>
-      </c>
-      <c r="J8">
-        <v>13</v>
-      </c>
-      <c r="K8">
-        <v>43</v>
-      </c>
-      <c r="L8" s="4">
-        <v>3.31</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8">
-        <v>3</v>
-      </c>
-      <c r="O8" s="11">
-        <f>56/217*100</f>
-        <v>25.806451612903224</v>
-      </c>
-      <c r="P8" s="11">
-        <f>904/2887*100</f>
-        <v>31.312781434014546</v>
-      </c>
-      <c r="Q8" s="11">
-        <f>8/25*100</f>
-        <v>32</v>
-      </c>
-      <c r="R8" s="11">
-        <f>(8+904)/(2887+25)*100</f>
-        <v>31.318681318681318</v>
-      </c>
-      <c r="S8" s="4">
-        <f>44/262*100</f>
-        <v>16.793893129770993</v>
-      </c>
-      <c r="T8" s="7">
-        <v>36349</v>
-      </c>
-      <c r="U8" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>21.783561643835615</v>
-      </c>
-      <c r="V8" s="11">
-        <f>5*12+9</f>
-        <v>69</v>
-      </c>
-      <c r="W8" s="11">
-        <v>178</v>
-      </c>
-      <c r="X8" s="11">
-        <v>10</v>
-      </c>
-      <c r="Y8" s="11">
-        <v>521</v>
-      </c>
-      <c r="Z8" s="4">
-        <v>73.099999999999994</v>
-      </c>
-      <c r="AA8" s="4">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>7.31</v>
-      </c>
-      <c r="AB8" s="15">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.1403071017274472</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
@@ -3800,19 +3793,19 @@
       <c r="N9">
         <v>1</v>
       </c>
-      <c r="O9" s="11">
+      <c r="O9" s="10">
         <f>101/365*100</f>
         <v>27.671232876712327</v>
       </c>
-      <c r="P9" s="11">
+      <c r="P9" s="10">
         <f>1275/4365*100</f>
         <v>29.209621993127151</v>
       </c>
-      <c r="Q9" s="11">
+      <c r="Q9" s="10">
         <f>11/35*100</f>
         <v>31.428571428571427</v>
       </c>
-      <c r="R9" s="11">
+      <c r="R9" s="10">
         <f>(11+1275)/(4365+35)*100</f>
         <v>29.22727272727273</v>
       </c>
@@ -3823,20 +3816,20 @@
         <v>35708</v>
       </c>
       <c r="U9" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>23.539726027397261</v>
-      </c>
-      <c r="V9" s="11">
+        <f ca="1">((TODAY()-T9)/365)-1</f>
+        <v>25.583561643835615</v>
+      </c>
+      <c r="V9" s="10">
         <f>6*12+4</f>
         <v>76</v>
       </c>
-      <c r="W9" s="11">
+      <c r="W9" s="10">
         <v>223</v>
       </c>
-      <c r="X9" s="11">
+      <c r="X9" s="10">
         <v>13</v>
       </c>
-      <c r="Y9" s="11">
+      <c r="Y9" s="10">
         <v>700</v>
       </c>
       <c r="Z9" s="4">
@@ -3846,7 +3839,7 @@
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
         <v>6.0692307692307699</v>
       </c>
-      <c r="AB9" s="15">
+      <c r="AB9" s="13">
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
         <v>0.11271428571428573</v>
       </c>
@@ -3894,19 +3887,19 @@
       <c r="N10">
         <v>1</v>
       </c>
-      <c r="O10" s="11">
+      <c r="O10" s="10">
         <f>56/257*100</f>
         <v>21.789883268482491</v>
       </c>
-      <c r="P10" s="11">
+      <c r="P10" s="10">
         <f>764/2858*100</f>
         <v>26.731980405878236</v>
       </c>
-      <c r="Q10" s="11">
+      <c r="Q10" s="10">
         <f>4/18*100</f>
         <v>22.222222222222221</v>
       </c>
-      <c r="R10" s="11">
+      <c r="R10" s="10">
         <f>(4+764)/(2858+18)*100</f>
         <v>26.703755215577189</v>
       </c>
@@ -3917,20 +3910,20 @@
         <v>36073</v>
       </c>
       <c r="U10" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>22.539726027397261</v>
-      </c>
-      <c r="V10" s="11">
+        <f ca="1">((TODAY()-T10)/365)-1</f>
+        <v>24.583561643835615</v>
+      </c>
+      <c r="V10" s="10">
         <f>6*12+1</f>
         <v>73</v>
       </c>
-      <c r="W10" s="11">
+      <c r="W10" s="10">
         <v>227</v>
       </c>
-      <c r="X10" s="11">
+      <c r="X10" s="10">
         <v>12</v>
       </c>
-      <c r="Y10" s="11">
+      <c r="Y10" s="10">
         <v>585</v>
       </c>
       <c r="Z10" s="4">
@@ -3940,855 +3933,856 @@
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
         <v>10.674999999999999</v>
       </c>
-      <c r="AB10" s="15">
+      <c r="AB10" s="13">
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
         <v>0.21897435897435896</v>
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C11">
-        <v>151</v>
+        <v>46</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E11" s="1">
         <v>13</v>
       </c>
       <c r="F11">
+        <v>56</v>
+      </c>
+      <c r="G11">
+        <v>904</v>
+      </c>
+      <c r="H11" s="4">
+        <v>16.14</v>
+      </c>
+      <c r="I11">
+        <v>8</v>
+      </c>
+      <c r="J11">
+        <v>13</v>
+      </c>
+      <c r="K11">
+        <v>43</v>
+      </c>
+      <c r="L11" s="4">
+        <v>3.31</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <v>3</v>
+      </c>
+      <c r="O11" s="10">
+        <f>56/217*100</f>
+        <v>25.806451612903224</v>
+      </c>
+      <c r="P11" s="10">
+        <f>904/2887*100</f>
+        <v>31.312781434014546</v>
+      </c>
+      <c r="Q11" s="10">
+        <f>8/25*100</f>
+        <v>32</v>
+      </c>
+      <c r="R11" s="10">
+        <f>(8+904)/(2887+25)*100</f>
+        <v>31.318681318681318</v>
+      </c>
+      <c r="S11" s="4">
+        <f>44/262*100</f>
+        <v>16.793893129770993</v>
+      </c>
+      <c r="T11" s="7">
+        <v>36349</v>
+      </c>
+      <c r="U11" s="5">
+        <f ca="1">((TODAY()-T11)/365)-1</f>
+        <v>23.827397260273973</v>
+      </c>
+      <c r="V11" s="10">
+        <f>5*12+9</f>
+        <v>69</v>
+      </c>
+      <c r="W11" s="10">
+        <v>178</v>
+      </c>
+      <c r="X11" s="10">
+        <v>10</v>
+      </c>
+      <c r="Y11" s="10">
+        <v>521</v>
+      </c>
+      <c r="Z11" s="4">
+        <v>73.099999999999994</v>
+      </c>
+      <c r="AA11" s="4">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
+        <v>7.31</v>
+      </c>
+      <c r="AB11" s="13">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
+        <v>0.1403071017274472</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12">
+        <v>49</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E12" s="1">
+        <v>13</v>
+      </c>
+      <c r="F12">
+        <v>66</v>
+      </c>
+      <c r="G12">
+        <v>1037</v>
+      </c>
+      <c r="H12" s="4">
+        <v>15.71</v>
+      </c>
+      <c r="I12">
+        <v>13</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12" s="10">
+        <f>66/253*100</f>
+        <v>26.086956521739129</v>
+      </c>
+      <c r="P12" s="10">
+        <f>1037/3278*100</f>
+        <v>31.63514338010982</v>
+      </c>
+      <c r="Q12" s="10">
+        <f>13/37*100</f>
+        <v>35.135135135135137</v>
+      </c>
+      <c r="R12" s="10">
+        <f>(13+1037)/(3278+37)*100</f>
+        <v>31.674208144796378</v>
+      </c>
+      <c r="S12" s="4">
+        <v>17.056000000000001</v>
+      </c>
+      <c r="T12" s="7">
+        <v>35983</v>
+      </c>
+      <c r="U12" s="5">
+        <f ca="1">((TODAY()-T12)/365)-1</f>
+        <v>24.830136986301369</v>
+      </c>
+      <c r="V12" s="10">
+        <f>6*12+4</f>
+        <v>76</v>
+      </c>
+      <c r="W12" s="10">
+        <v>238</v>
+      </c>
+      <c r="X12" s="10">
+        <v>14</v>
+      </c>
+      <c r="Y12" s="10">
+        <v>692</v>
+      </c>
+      <c r="Z12" s="4">
+        <v>181.9</v>
+      </c>
+      <c r="AA12" s="4">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
+        <v>12.992857142857144</v>
+      </c>
+      <c r="AB12" s="13">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
+        <v>0.26286127167630058</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13">
+        <v>57</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E13" s="1">
+        <v>13</v>
+      </c>
+      <c r="F13">
+        <v>49</v>
+      </c>
+      <c r="G13">
+        <v>657</v>
+      </c>
+      <c r="H13" s="4">
+        <v>13.41</v>
+      </c>
+      <c r="I13">
+        <v>6</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
+      </c>
+      <c r="K13">
+        <v>7</v>
+      </c>
+      <c r="L13" s="4">
+        <v>7</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13" s="10">
+        <f>49/317*100</f>
+        <v>15.457413249211358</v>
+      </c>
+      <c r="P13" s="10">
+        <f>657/3910*100</f>
+        <v>16.803069053708438</v>
+      </c>
+      <c r="Q13" s="10">
+        <f>6/33*100</f>
+        <v>18.181818181818183</v>
+      </c>
+      <c r="R13" s="10">
+        <f>(6+657)/(3910+33)*100</f>
+        <v>16.814608166370785</v>
+      </c>
+      <c r="S13" s="4">
+        <v>19.591999999999999</v>
+      </c>
+      <c r="T13" s="7">
+        <v>35272</v>
+      </c>
+      <c r="U13" s="5">
+        <f ca="1">((TODAY()-T13)/365)-1</f>
+        <v>26.778082191780822</v>
+      </c>
+      <c r="V13" s="10">
+        <f>6*12+1</f>
+        <v>73</v>
+      </c>
+      <c r="W13" s="10">
+        <v>200</v>
+      </c>
+      <c r="X13" s="10">
+        <v>2.79</v>
+      </c>
+      <c r="Y13" s="10">
+        <v>256</v>
+      </c>
+      <c r="Z13" s="4">
+        <v>36.4</v>
+      </c>
+      <c r="AA13" s="4">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
+        <v>13.046594982078853</v>
+      </c>
+      <c r="AB13" s="13">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
+        <v>0.14218749999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14">
+        <v>59</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E14" s="1">
+        <v>14</v>
+      </c>
+      <c r="F14">
+        <v>66</v>
+      </c>
+      <c r="G14">
+        <v>1020</v>
+      </c>
+      <c r="H14" s="4">
+        <v>15.45</v>
+      </c>
+      <c r="I14">
+        <v>12</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14" s="4">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <v>2</v>
+      </c>
+      <c r="O14" s="10">
+        <f>66/277*100</f>
+        <v>23.826714801444044</v>
+      </c>
+      <c r="P14" s="10">
+        <f>1020/3571*100</f>
+        <v>28.563427611313358</v>
+      </c>
+      <c r="Q14" s="10">
+        <f>12/24*100</f>
+        <v>50</v>
+      </c>
+      <c r="R14" s="10">
+        <f>(12+1020)/(3571+24)*100</f>
+        <v>28.70653685674548</v>
+      </c>
+      <c r="S14" s="4">
+        <v>51.3</v>
+      </c>
+      <c r="T14" s="7">
+        <v>35713</v>
+      </c>
+      <c r="U14" s="5">
+        <f ca="1">((TODAY()-T14)/365)-1</f>
+        <v>25.56986301369863</v>
+      </c>
+      <c r="V14" s="10">
+        <f>6*12+3</f>
+        <v>75</v>
+      </c>
+      <c r="W14" s="10">
+        <v>207</v>
+      </c>
+      <c r="X14" s="10">
+        <v>8</v>
+      </c>
+      <c r="Y14" s="10">
+        <v>439</v>
+      </c>
+      <c r="Z14" s="4">
+        <v>49.2</v>
+      </c>
+      <c r="AA14" s="4">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
+        <v>6.15</v>
+      </c>
+      <c r="AB14" s="13">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
+        <v>0.11207289293849659</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15">
+        <v>81</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E15" s="1">
+        <v>10</v>
+      </c>
+      <c r="F15">
+        <v>71</v>
+      </c>
+      <c r="G15">
+        <v>816</v>
+      </c>
+      <c r="H15" s="4">
+        <v>11.49</v>
+      </c>
+      <c r="I15">
+        <v>6</v>
+      </c>
+      <c r="J15">
+        <v>2</v>
+      </c>
+      <c r="K15">
+        <v>22</v>
+      </c>
+      <c r="L15" s="4">
+        <v>11</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15" s="10">
+        <f>71/268*100</f>
+        <v>26.492537313432834</v>
+      </c>
+      <c r="P15" s="10">
+        <f>816/2667*100</f>
+        <v>30.596175478065241</v>
+      </c>
+      <c r="Q15" s="10">
+        <f>6/12*100</f>
+        <v>50</v>
+      </c>
+      <c r="R15" s="10">
+        <f>(6+816)/(2667+12)*100</f>
+        <v>30.683090705487121</v>
+      </c>
+      <c r="S15" s="4">
+        <v>47.41</v>
+      </c>
+      <c r="T15" s="7">
+        <v>36112</v>
+      </c>
+      <c r="U15" s="5">
+        <f ca="1">((TODAY()-T15)/365)-1</f>
+        <v>24.476712328767125</v>
+      </c>
+      <c r="V15" s="10">
+        <f>6*12+3</f>
+        <v>75</v>
+      </c>
+      <c r="W15" s="10">
+        <v>212</v>
+      </c>
+      <c r="X15" s="10">
+        <v>3</v>
+      </c>
+      <c r="Y15" s="10">
+        <v>259</v>
+      </c>
+      <c r="Z15" s="4">
+        <v>30.8</v>
+      </c>
+      <c r="AA15" s="4">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
+        <v>10.266666666666667</v>
+      </c>
+      <c r="AB15" s="13">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
+        <v>0.11891891891891893</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16">
+        <v>92</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E16" s="1">
+        <v>13</v>
+      </c>
+      <c r="F16">
+        <v>106</v>
+      </c>
+      <c r="G16">
+        <v>1386</v>
+      </c>
+      <c r="H16" s="4">
+        <v>13.08</v>
+      </c>
+      <c r="I16">
+        <v>9</v>
+      </c>
+      <c r="J16">
+        <v>10</v>
+      </c>
+      <c r="K16">
+        <v>24</v>
+      </c>
+      <c r="L16" s="4">
+        <v>2.4</v>
+      </c>
+      <c r="M16">
+        <v>1</v>
+      </c>
+      <c r="N16" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="O16" s="10">
+        <f>106/306*100</f>
+        <v>34.640522875816991</v>
+      </c>
+      <c r="P16" s="10">
+        <f>1386/3761*100</f>
+        <v>36.851901090135605</v>
+      </c>
+      <c r="Q16" s="10">
+        <f>9/32*100</f>
+        <v>28.125</v>
+      </c>
+      <c r="R16" s="10">
+        <f>(1386+9)/(3761+32)*100</f>
+        <v>36.778275771157389</v>
+      </c>
+      <c r="S16" s="14">
+        <v>20.879000000000001</v>
+      </c>
+      <c r="T16" s="8">
+        <v>35685</v>
+      </c>
+      <c r="U16" s="5">
+        <f ca="1">((TODAY()-T16)/365)-1</f>
+        <v>25.646575342465752</v>
+      </c>
+      <c r="V16" s="10">
+        <f>5*12+11</f>
+        <v>71</v>
+      </c>
+      <c r="W16" s="10">
+        <v>210</v>
+      </c>
+      <c r="X16" s="10">
+        <v>6</v>
+      </c>
+      <c r="Y16" s="10">
+        <v>347</v>
+      </c>
+      <c r="Z16" s="4">
+        <v>43.1</v>
+      </c>
+      <c r="AA16" s="4">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
+        <v>7.1833333333333336</v>
+      </c>
+      <c r="AB16" s="13">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
+        <v>0.12420749279538905</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17">
+        <v>128</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E17" s="1">
+        <v>12</v>
+      </c>
+      <c r="F17">
+        <v>72</v>
+      </c>
+      <c r="G17">
+        <v>1241</v>
+      </c>
+      <c r="H17" s="4">
+        <v>17.239999999999998</v>
+      </c>
+      <c r="I17">
+        <v>12</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17" s="4">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17" s="10">
+        <f>72/271*100</f>
+        <v>26.568265682656829</v>
+      </c>
+      <c r="P17" s="10">
+        <f>1241/4117*100</f>
+        <v>30.143308234151078</v>
+      </c>
+      <c r="Q17" s="10">
+        <f>12/36*100</f>
+        <v>33.333333333333329</v>
+      </c>
+      <c r="R17" s="10">
+        <f>(1241+12)/(4117+36)*100</f>
+        <v>30.170960751264147</v>
+      </c>
+      <c r="S17" s="4">
+        <v>11.18</v>
+      </c>
+      <c r="T17" s="7">
+        <v>36251</v>
+      </c>
+      <c r="U17" s="5">
+        <f ca="1">((TODAY()-T17)/365)-1</f>
+        <v>24.095890410958905</v>
+      </c>
+      <c r="V17" s="10">
+        <f>6*12+2</f>
+        <v>74</v>
+      </c>
+      <c r="W17" s="10">
+        <v>210</v>
+      </c>
+      <c r="X17" s="10">
+        <v>15</v>
+      </c>
+      <c r="Y17" s="10">
+        <v>797</v>
+      </c>
+      <c r="Z17" s="4">
+        <v>118.4</v>
+      </c>
+      <c r="AA17" s="4">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
+        <v>7.8933333333333335</v>
+      </c>
+      <c r="AB17" s="13">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
+        <v>0.14855708908406526</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C18">
+        <v>142</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E18" s="1">
+        <v>13</v>
+      </c>
+      <c r="F18">
+        <v>79</v>
+      </c>
+      <c r="G18">
+        <v>1396</v>
+      </c>
+      <c r="H18" s="4">
+        <v>17.670000000000002</v>
+      </c>
+      <c r="I18">
+        <v>10</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18" s="4">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18" t="s">
+        <v>39</v>
+      </c>
+      <c r="O18" s="10">
+        <f>79/257*100</f>
+        <v>30.739299610894943</v>
+      </c>
+      <c r="P18" s="10">
+        <f>1396/3756*100</f>
+        <v>37.167199148029816</v>
+      </c>
+      <c r="Q18" s="10">
+        <f>10/29*100</f>
+        <v>34.482758620689658</v>
+      </c>
+      <c r="R18" s="10">
+        <f>(10+1396)/(29+3756)*100</f>
+        <v>37.146631439894321</v>
+      </c>
+      <c r="S18" s="4">
+        <v>47.037999999999997</v>
+      </c>
+      <c r="T18" s="7">
+        <v>35896</v>
+      </c>
+      <c r="U18" s="5">
+        <f ca="1">((TODAY()-T18)/365)-1</f>
+        <v>25.068493150684933</v>
+      </c>
+      <c r="V18" s="10">
+        <f>6*12+4</f>
+        <v>76</v>
+      </c>
+      <c r="W18" s="10">
+        <v>223</v>
+      </c>
+      <c r="X18" s="10">
+        <v>2</v>
+      </c>
+      <c r="Y18" s="10">
+        <v>124</v>
+      </c>
+      <c r="Z18" s="4">
+        <v>3</v>
+      </c>
+      <c r="AA18" s="4">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
+        <v>1.5</v>
+      </c>
+      <c r="AB18" s="13">
+        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
+        <v>2.4193548387096774E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19">
+        <v>151</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E19" s="1">
+        <v>13</v>
+      </c>
+      <c r="F19">
         <v>77</v>
       </c>
-      <c r="G11">
+      <c r="G19">
         <v>679</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H19" s="4">
         <v>8.82</v>
       </c>
-      <c r="I11">
+      <c r="I19">
         <v>7</v>
       </c>
-      <c r="J11">
+      <c r="J19">
         <v>8</v>
       </c>
-      <c r="K11">
+      <c r="K19">
         <v>42</v>
       </c>
-      <c r="L11" s="4">
+      <c r="L19" s="4">
         <v>5.25</v>
       </c>
-      <c r="M11">
-        <v>0</v>
-      </c>
-      <c r="N11">
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19">
         <v>1</v>
       </c>
-      <c r="O11" s="12">
+      <c r="O19" s="10">
         <f>77/337*100</f>
         <v>22.848664688427299</v>
       </c>
-      <c r="P11" s="12">
+      <c r="P19" s="10">
         <f>679/3748*100</f>
         <v>18.116328708644609</v>
       </c>
-      <c r="Q11" s="12">
+      <c r="Q19" s="10">
         <f>7/23*100</f>
         <v>30.434782608695656</v>
       </c>
-      <c r="R11" s="12">
+      <c r="R19" s="10">
         <f>(7+679)/(3748+23)*100</f>
         <v>18.191461150888358</v>
       </c>
-      <c r="S11" s="4">
+      <c r="S19" s="4">
         <v>16.61</v>
       </c>
-      <c r="T11" s="7">
+      <c r="T19" s="7">
         <v>35799</v>
       </c>
-      <c r="U11" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>23.290410958904111</v>
-      </c>
-      <c r="V11" s="11">
+      <c r="U19" s="5">
+        <f ca="1">((TODAY()-T19)/365)-1</f>
+        <v>25.334246575342465</v>
+      </c>
+      <c r="V19" s="10">
         <f>6*12</f>
         <v>72</v>
       </c>
-      <c r="W11" s="11">
+      <c r="W19" s="10">
         <v>224</v>
       </c>
-      <c r="X11" s="11">
+      <c r="X19" s="10">
         <v>0.81</v>
       </c>
-      <c r="Y11" s="11">
+      <c r="Y19" s="10">
         <v>27</v>
       </c>
-      <c r="Z11" s="4">
+      <c r="Z19" s="4">
         <v>8.9</v>
       </c>
-      <c r="AA11" s="4">
+      <c r="AA19" s="4">
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
         <v>10.987654320987653</v>
       </c>
-      <c r="AB11" s="15">
+      <c r="AB19" s="13">
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
         <v>0.32962962962962966</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12">
-        <v>57</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="E12" s="1">
-        <v>13</v>
-      </c>
-      <c r="F12">
-        <v>49</v>
-      </c>
-      <c r="G12">
-        <v>657</v>
-      </c>
-      <c r="H12" s="4">
-        <v>13.41</v>
-      </c>
-      <c r="I12">
-        <v>6</v>
-      </c>
-      <c r="J12">
-        <v>1</v>
-      </c>
-      <c r="K12">
-        <v>7</v>
-      </c>
-      <c r="L12" s="4">
-        <v>7</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="N12">
-        <v>0</v>
-      </c>
-      <c r="O12" s="11">
-        <f>49/317*100</f>
-        <v>15.457413249211358</v>
-      </c>
-      <c r="P12" s="11">
-        <f>657/3910*100</f>
-        <v>16.803069053708438</v>
-      </c>
-      <c r="Q12" s="11">
-        <f>6/33*100</f>
-        <v>18.181818181818183</v>
-      </c>
-      <c r="R12" s="11">
-        <f>(6+657)/(3910+33)*100</f>
-        <v>16.814608166370785</v>
-      </c>
-      <c r="S12" s="4">
-        <v>19.591999999999999</v>
-      </c>
-      <c r="T12" s="7">
-        <v>35272</v>
-      </c>
-      <c r="U12" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>24.734246575342464</v>
-      </c>
-      <c r="V12" s="11">
-        <f>6*12+1</f>
-        <v>73</v>
-      </c>
-      <c r="W12" s="11">
-        <v>200</v>
-      </c>
-      <c r="X12" s="11">
-        <v>2.79</v>
-      </c>
-      <c r="Y12" s="11">
-        <v>256</v>
-      </c>
-      <c r="Z12" s="4">
-        <v>36.4</v>
-      </c>
-      <c r="AA12" s="4">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>13.046594982078853</v>
-      </c>
-      <c r="AB12" s="15">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.14218749999999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13">
-        <v>12</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="E13" s="1">
-        <v>12</v>
-      </c>
-      <c r="F13">
-        <v>40</v>
-      </c>
-      <c r="G13">
-        <v>746</v>
-      </c>
-      <c r="H13" s="4">
-        <v>18.649999999999999</v>
-      </c>
-      <c r="I13">
-        <v>7</v>
-      </c>
-      <c r="J13">
-        <v>2</v>
-      </c>
-      <c r="K13">
-        <v>75</v>
-      </c>
-      <c r="L13" s="4">
-        <v>37.5</v>
-      </c>
-      <c r="M13">
-        <v>1</v>
-      </c>
-      <c r="N13">
-        <v>0</v>
-      </c>
-      <c r="O13" s="11">
-        <f>40/287*100</f>
-        <v>13.937282229965156</v>
-      </c>
-      <c r="P13" s="11">
-        <f>746/4449*100</f>
-        <v>16.767812991683524</v>
-      </c>
-      <c r="Q13" s="11">
-        <f>7/49*100</f>
-        <v>14.285714285714285</v>
-      </c>
-      <c r="R13" s="11">
-        <f>(746+7)/(4449+49)*100</f>
-        <v>16.740773677189864</v>
-      </c>
-      <c r="S13" s="4">
-        <v>47.41</v>
-      </c>
-      <c r="T13" s="7">
-        <v>36184</v>
-      </c>
-      <c r="U13" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>22.235616438356164</v>
-      </c>
-      <c r="V13" s="11">
-        <f>6*12</f>
-        <v>72</v>
-      </c>
-      <c r="W13" s="11">
-        <v>190</v>
-      </c>
-      <c r="X13" s="11">
-        <v>13</v>
-      </c>
-      <c r="Y13" s="11">
-        <v>581</v>
-      </c>
-      <c r="Z13" s="4">
-        <v>71.099999999999994</v>
-      </c>
-      <c r="AA13" s="4">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>5.4692307692307685</v>
-      </c>
-      <c r="AB13" s="15">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.12237521514629947</v>
-      </c>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C14">
-        <v>81</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="E14" s="1">
-        <v>10</v>
-      </c>
-      <c r="F14">
-        <v>71</v>
-      </c>
-      <c r="G14">
-        <v>816</v>
-      </c>
-      <c r="H14" s="4">
-        <v>11.49</v>
-      </c>
-      <c r="I14">
-        <v>6</v>
-      </c>
-      <c r="J14">
-        <v>2</v>
-      </c>
-      <c r="K14">
-        <v>22</v>
-      </c>
-      <c r="L14" s="4">
-        <v>11</v>
-      </c>
-      <c r="M14">
-        <v>0</v>
-      </c>
-      <c r="N14">
-        <v>0</v>
-      </c>
-      <c r="O14" s="11">
-        <f>71/268*100</f>
-        <v>26.492537313432834</v>
-      </c>
-      <c r="P14" s="11">
-        <f>816/2667*100</f>
-        <v>30.596175478065241</v>
-      </c>
-      <c r="Q14" s="11">
-        <f>6/12*100</f>
-        <v>50</v>
-      </c>
-      <c r="R14" s="11">
-        <f>(6+816)/(2667+12)*100</f>
-        <v>30.683090705487121</v>
-      </c>
-      <c r="S14" s="4">
-        <v>47.41</v>
-      </c>
-      <c r="T14" s="7">
-        <v>36112</v>
-      </c>
-      <c r="U14" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>22.432876712328767</v>
-      </c>
-      <c r="V14" s="11">
-        <f>6*12+3</f>
-        <v>75</v>
-      </c>
-      <c r="W14" s="11">
-        <v>212</v>
-      </c>
-      <c r="X14" s="11">
-        <v>3</v>
-      </c>
-      <c r="Y14" s="11">
-        <v>259</v>
-      </c>
-      <c r="Z14" s="4">
-        <v>30.8</v>
-      </c>
-      <c r="AA14" s="4">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>10.266666666666667</v>
-      </c>
-      <c r="AB14" s="15">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.11891891891891893</v>
-      </c>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15">
-        <v>22</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E15" s="1">
-        <v>15</v>
-      </c>
-      <c r="F15">
-        <v>111</v>
-      </c>
-      <c r="G15">
-        <v>1540</v>
-      </c>
-      <c r="H15" s="4">
-        <v>13.87</v>
-      </c>
-      <c r="I15">
-        <v>18</v>
-      </c>
-      <c r="J15">
-        <v>0</v>
-      </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15" s="4">
-        <v>0</v>
-      </c>
-      <c r="M15">
-        <v>0</v>
-      </c>
-      <c r="N15">
-        <v>0</v>
-      </c>
-      <c r="O15" s="11">
-        <f>111/426*100</f>
-        <v>26.056338028169012</v>
-      </c>
-      <c r="P15" s="11">
-        <f>1540/6024*100</f>
-        <v>25.564409030544489</v>
-      </c>
-      <c r="Q15" s="11">
-        <f>18/61*100</f>
-        <v>29.508196721311474</v>
-      </c>
-      <c r="R15" s="11">
-        <f>(18+1540)/(6024+61)*100</f>
-        <v>25.603944124897289</v>
-      </c>
-      <c r="S15" s="4">
-        <v>52.63</v>
-      </c>
-      <c r="T15" s="7">
-        <v>36176</v>
-      </c>
-      <c r="U15" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>22.257534246575343</v>
-      </c>
-      <c r="V15" s="11">
-        <f>6*12+1</f>
-        <v>73</v>
-      </c>
-      <c r="W15" s="11">
-        <v>202</v>
-      </c>
-      <c r="X15" s="11">
-        <v>16</v>
-      </c>
-      <c r="Y15" s="11">
-        <v>886</v>
-      </c>
-      <c r="Z15" s="4">
-        <v>229.2</v>
-      </c>
-      <c r="AA15" s="4">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>14.324999999999999</v>
-      </c>
-      <c r="AB15" s="15">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.2586907449209932</v>
-      </c>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C16">
-        <v>59</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="E16" s="1">
-        <v>14</v>
-      </c>
-      <c r="F16">
-        <v>66</v>
-      </c>
-      <c r="G16">
-        <v>1020</v>
-      </c>
-      <c r="H16" s="4">
-        <v>15.45</v>
-      </c>
-      <c r="I16">
-        <v>12</v>
-      </c>
-      <c r="J16">
-        <v>0</v>
-      </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
-      <c r="L16" s="4">
-        <v>0</v>
-      </c>
-      <c r="M16">
-        <v>0</v>
-      </c>
-      <c r="N16">
-        <v>2</v>
-      </c>
-      <c r="O16" s="11">
-        <f>66/277*100</f>
-        <v>23.826714801444044</v>
-      </c>
-      <c r="P16" s="11">
-        <f>1020/3571*100</f>
-        <v>28.563427611313358</v>
-      </c>
-      <c r="Q16" s="11">
-        <f>12/24*100</f>
-        <v>50</v>
-      </c>
-      <c r="R16" s="11">
-        <f>(12+1020)/(3571+24)*100</f>
-        <v>28.70653685674548</v>
-      </c>
-      <c r="S16" s="4">
-        <v>51.3</v>
-      </c>
-      <c r="T16" s="7">
-        <v>35713</v>
-      </c>
-      <c r="U16" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>23.526027397260275</v>
-      </c>
-      <c r="V16" s="11">
-        <f>6*12+3</f>
-        <v>75</v>
-      </c>
-      <c r="W16" s="11">
-        <v>207</v>
-      </c>
-      <c r="X16" s="11">
-        <v>8</v>
-      </c>
-      <c r="Y16" s="11">
-        <v>439</v>
-      </c>
-      <c r="Z16" s="4">
-        <v>49.2</v>
-      </c>
-      <c r="AA16" s="4">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>6.15</v>
-      </c>
-      <c r="AB16" s="15">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.11207289293849659</v>
-      </c>
-    </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C17">
-        <v>21</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E17" s="1">
-        <v>12</v>
-      </c>
-      <c r="F17">
-        <v>43</v>
-      </c>
-      <c r="G17">
-        <v>611</v>
-      </c>
-      <c r="H17" s="4">
-        <v>14.21</v>
-      </c>
-      <c r="I17">
-        <v>5</v>
-      </c>
-      <c r="J17">
-        <v>14</v>
-      </c>
-      <c r="K17">
-        <v>89</v>
-      </c>
-      <c r="L17" s="4">
-        <v>6.36</v>
-      </c>
-      <c r="M17">
-        <v>0</v>
-      </c>
-      <c r="N17">
-        <v>6</v>
-      </c>
-      <c r="O17" s="11">
-        <f>43/211*100</f>
-        <v>20.379146919431278</v>
-      </c>
-      <c r="P17" s="11">
-        <f>611/2444*100</f>
-        <v>25</v>
-      </c>
-      <c r="Q17" s="11">
-        <f>5/15*100</f>
-        <v>33.333333333333329</v>
-      </c>
-      <c r="R17" s="11">
-        <f>(5+611)/(2444+15)*100</f>
-        <v>25.050833672224481</v>
-      </c>
-      <c r="S17" s="4">
-        <v>42.23</v>
-      </c>
-      <c r="T17" s="7">
-        <v>36161</v>
-      </c>
-      <c r="U17" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>22.298630136986301</v>
-      </c>
-      <c r="V17" s="11">
-        <f>5*12+11</f>
-        <v>71</v>
-      </c>
-      <c r="W17" s="11">
-        <v>197</v>
-      </c>
-      <c r="X17" s="11">
-        <v>10</v>
-      </c>
-      <c r="Y17" s="11">
-        <v>511</v>
-      </c>
-      <c r="Z17" s="4">
-        <v>70.7</v>
-      </c>
-      <c r="AA17" s="4">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>7.07</v>
-      </c>
-      <c r="AB17" s="15">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.13835616438356166</v>
-      </c>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C18">
-        <v>49</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E18" s="1">
-        <v>13</v>
-      </c>
-      <c r="F18">
-        <v>66</v>
-      </c>
-      <c r="G18">
-        <v>1037</v>
-      </c>
-      <c r="H18" s="4">
-        <v>15.71</v>
-      </c>
-      <c r="I18">
-        <v>13</v>
-      </c>
-      <c r="J18">
-        <v>0</v>
-      </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
-        <v>0</v>
-      </c>
-      <c r="M18">
-        <v>0</v>
-      </c>
-      <c r="N18">
-        <v>0</v>
-      </c>
-      <c r="O18" s="11">
-        <f>66/253*100</f>
-        <v>26.086956521739129</v>
-      </c>
-      <c r="P18" s="11">
-        <f>1037/3278*100</f>
-        <v>31.63514338010982</v>
-      </c>
-      <c r="Q18" s="11">
-        <f>13/37*100</f>
-        <v>35.135135135135137</v>
-      </c>
-      <c r="R18" s="11">
-        <f>(13+1037)/(3278+37)*100</f>
-        <v>31.674208144796378</v>
-      </c>
-      <c r="S18" s="4">
-        <v>17.056000000000001</v>
-      </c>
-      <c r="T18" s="7">
-        <v>35983</v>
-      </c>
-      <c r="U18" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>22.786301369863015</v>
-      </c>
-      <c r="V18" s="11">
-        <f>6*12+4</f>
-        <v>76</v>
-      </c>
-      <c r="W18" s="11">
-        <v>238</v>
-      </c>
-      <c r="X18" s="11">
-        <v>14</v>
-      </c>
-      <c r="Y18" s="11">
-        <v>692</v>
-      </c>
-      <c r="Z18" s="4">
-        <v>181.9</v>
-      </c>
-      <c r="AA18" s="4">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>12.992857142857144</v>
-      </c>
-      <c r="AB18" s="15">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.26286127167630058</v>
-      </c>
-    </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C19">
-        <v>25</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E19" s="1">
-        <v>12</v>
-      </c>
-      <c r="F19">
-        <v>65</v>
-      </c>
-      <c r="G19">
-        <v>1192</v>
-      </c>
-      <c r="H19" s="4">
-        <v>18.34</v>
-      </c>
-      <c r="I19">
-        <v>8</v>
-      </c>
-      <c r="J19">
-        <v>1</v>
-      </c>
-      <c r="K19">
-        <v>6</v>
-      </c>
-      <c r="L19" s="4">
-        <v>6</v>
-      </c>
-      <c r="M19">
-        <v>0</v>
-      </c>
-      <c r="N19">
-        <v>1</v>
-      </c>
-      <c r="O19" s="11">
-        <f>65/233*100</f>
-        <v>27.896995708154503</v>
-      </c>
-      <c r="P19" s="11">
-        <f>1192/3235*100</f>
-        <v>36.84698608964451</v>
-      </c>
-      <c r="Q19" s="11">
-        <f>8/21*100</f>
-        <v>38.095238095238095</v>
-      </c>
-      <c r="R19" s="11">
-        <f>(8+1192)/(3235+21)*100</f>
-        <v>36.855036855036857</v>
-      </c>
-      <c r="S19" s="4">
-        <v>48.927</v>
-      </c>
-      <c r="T19" s="7">
-        <v>35871</v>
-      </c>
-      <c r="U19" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>23.093150684931508</v>
-      </c>
-      <c r="V19" s="11">
-        <f>6*12</f>
-        <v>72</v>
-      </c>
-      <c r="W19" s="11">
-        <v>200</v>
-      </c>
-      <c r="X19" s="11">
-        <v>12</v>
-      </c>
-      <c r="Y19" s="11">
-        <v>728</v>
-      </c>
-      <c r="Z19" s="4">
-        <v>154.5</v>
-      </c>
-      <c r="AA19" s="4">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>12.875</v>
-      </c>
-      <c r="AB19" s="15">
-        <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>0.21222527472527472</v>
       </c>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.25">
@@ -4834,19 +4828,19 @@
       <c r="N20">
         <v>2</v>
       </c>
-      <c r="O20" s="12">
+      <c r="O20" s="10">
         <f>86/212*100</f>
         <v>40.566037735849058</v>
       </c>
-      <c r="P20" s="12">
+      <c r="P20" s="10">
         <f>1318/3298*100</f>
         <v>39.963614311704063</v>
       </c>
-      <c r="Q20" s="12">
+      <c r="Q20" s="10">
         <f>13/31*100</f>
         <v>41.935483870967744</v>
       </c>
-      <c r="R20" s="12">
+      <c r="R20" s="10">
         <f>(13+1318)/(3293+31)*100</f>
         <v>40.042117930204576</v>
       </c>
@@ -4857,20 +4851,20 @@
         <v>36032</v>
       </c>
       <c r="U20" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>22.652054794520549</v>
-      </c>
-      <c r="V20" s="11">
+        <f ca="1">((TODAY()-T20)/365)-1</f>
+        <v>24.695890410958903</v>
+      </c>
+      <c r="V20" s="10">
         <f>6*12+2</f>
         <v>74</v>
       </c>
-      <c r="W20" s="11">
+      <c r="W20" s="10">
         <v>206</v>
       </c>
-      <c r="X20" s="11">
+      <c r="X20" s="10">
         <v>2.5</v>
       </c>
-      <c r="Y20" s="11">
+      <c r="Y20" s="10">
         <v>264</v>
       </c>
       <c r="Z20" s="4">
@@ -4880,38 +4874,39 @@
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
         <v>13.959999999999999</v>
       </c>
-      <c r="AB20" s="15">
+      <c r="AB20" s="13">
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
         <v>0.1321969696969697</v>
       </c>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>55</v>
+        <v>127</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>74</v>
+        <v>128</v>
       </c>
       <c r="C21">
-        <v>142</v>
+        <v>173</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>96</v>
+        <v>129</v>
       </c>
       <c r="E21" s="1">
         <v>13</v>
       </c>
       <c r="F21">
-        <v>79</v>
+        <v>48</v>
       </c>
       <c r="G21">
-        <v>1396</v>
+        <v>713</v>
       </c>
       <c r="H21" s="4">
-        <v>17.670000000000002</v>
+        <f>Table3[[#This Row],[Rec.Yds]]/Table3[[#This Row],[Receptions]]</f>
+        <v>14.854166666666666</v>
       </c>
       <c r="I21">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J21">
         <v>0</v>
@@ -4925,58 +4920,59 @@
       <c r="M21">
         <v>0</v>
       </c>
-      <c r="N21" t="s">
-        <v>39</v>
-      </c>
-      <c r="O21" s="12">
-        <f>79/257*100</f>
-        <v>30.739299610894943</v>
-      </c>
-      <c r="P21" s="12">
-        <f>1396/3756*100</f>
-        <v>37.167199148029816</v>
-      </c>
-      <c r="Q21" s="12">
-        <f>10/29*100</f>
-        <v>34.482758620689658</v>
-      </c>
-      <c r="R21" s="12">
-        <f>(10+1396)/(29+3756)*100</f>
-        <v>37.146631439894321</v>
+      <c r="N21">
+        <v>0</v>
+      </c>
+      <c r="O21" s="10">
+        <f>48/197*100</f>
+        <v>24.36548223350254</v>
+      </c>
+      <c r="P21" s="10">
+        <f>713/2679*100</f>
+        <v>26.614408361328856</v>
+      </c>
+      <c r="Q21" s="10">
+        <f>5/19*100</f>
+        <v>26.315789473684209</v>
+      </c>
+      <c r="R21" s="10">
+        <f>(5+713)/(19+2679)*100</f>
+        <v>26.612305411415864</v>
       </c>
       <c r="S21" s="4">
-        <v>47.037999999999997</v>
+        <f>48/350*100</f>
+        <v>13.714285714285715</v>
       </c>
       <c r="T21" s="7">
-        <v>35896</v>
+        <v>35732</v>
       </c>
       <c r="U21" s="5">
-        <f t="shared" ca="1" si="0"/>
-        <v>23.024657534246575</v>
-      </c>
-      <c r="V21" s="11">
-        <f>6*12+4</f>
-        <v>76</v>
-      </c>
-      <c r="W21" s="11">
-        <v>223</v>
-      </c>
-      <c r="X21" s="11">
-        <v>2</v>
-      </c>
-      <c r="Y21" s="11">
-        <v>124</v>
+        <f ca="1">((TODAY()-T21)/365)-1</f>
+        <v>25.517808219178082</v>
+      </c>
+      <c r="V21" s="10">
+        <f>5*12+11</f>
+        <v>71</v>
+      </c>
+      <c r="W21" s="10">
+        <v>174</v>
+      </c>
+      <c r="X21" s="10">
+        <v>15</v>
+      </c>
+      <c r="Y21" s="10">
+        <v>781</v>
       </c>
       <c r="Z21" s="4">
-        <v>3</v>
+        <v>120.6</v>
       </c>
       <c r="AA21" s="4">
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[NFL.Games]]</f>
-        <v>1.5</v>
-      </c>
-      <c r="AB21" s="15">
+        <v>8.0399999999999991</v>
+      </c>
+      <c r="AB21" s="13">
         <f>Table3[[#This Row],[FP]]/Table3[[#This Row],[Snaps]]</f>
-        <v>2.4193548387096774E-2</v>
+        <v>0.15441741357234315</v>
       </c>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.25">

</xml_diff>